<commit_message>
Successfully test Docker grading flow on student cuongnhhe186494
Co-authored-by: bstHoang <139115555+bstHoang@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/1/student/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
+++ b/Submit/Results/1/student/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
@@ -120,56 +120,25 @@
     <x:t>NetworkResult</x:t>
   </x:si>
   <x:si>
-    <x:t>05:26:21.963</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TCP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>172.18.0.3:60058</x:t>
-  </x:si>
-  <x:si>
-    <x:t>172.18.0.2:8000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SYN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Connection Request</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Client</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Server</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SYN, ACK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Connection Accepted</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>05:26:21.964</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACK, PSH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Data Transfer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1 + 2
-</x:t>
-  </x:si>
-  <x:si>
-    <x:t>05:26:21.966</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3</x:t>
+    <x:t>Flags=SYN, Data=, From=Client</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FAIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Network flow not found</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Flags=SYN, ACK, Data=, From=Server</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Flags=ACK, Data=, From=Client</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Flags=PSH, ACK, Data=1 + 2, From=Client</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Flags=ACK, Data=, From=Server</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -772,15 +741,16 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:P15"/>
+  <x:dimension ref="A1:Q6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="5.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.853482" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="8.567768" style="0" customWidth="1"/>
-    <x:col min="4" max="5" width="15.853482" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.139196" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="19.996339" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="6.853482" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="11.139196" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="37.139196" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="5.424911" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="4.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="10.853482" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="8.853482" style="0" customWidth="1"/>
@@ -790,9 +760,10 @@
     <x:col min="14" max="14" width="10.567768" style="0" customWidth="1"/>
     <x:col min="15" max="15" width="9.140625" style="0" customWidth="1"/>
     <x:col min="16" max="16" width="14.139196" style="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:16" s="1" customFormat="1">
+    <x:row r="1" spans="1:17" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -839,632 +810,74 @@
         <x:v>32</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:16">
+    <x:row r="2" spans="1:17">
       <x:c r="A2" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B2" s="0" t="s">
+      <x:c r="F2" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="C2" s="0" t="s">
+      <x:c r="P2" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="D2" s="0" t="s">
+      <x:c r="Q2" s="0" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F2" s="0" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G2" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="I2" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J2" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K2" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P2" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:16">
+    </x:row>
+    <x:row r="3" spans="1:17">
       <x:c r="A3" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
+      <x:c r="F3" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="P3" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s">
+      <x:c r="Q3" s="0" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="I3" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J3" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K3" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L3" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M3" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N3" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P3" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:16">
+    </x:row>
+    <x:row r="4" spans="1:17">
       <x:c r="A4" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
+      <x:c r="F4" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="P4" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
+      <x:c r="Q4" s="0" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="I4" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J4" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="K4" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L4" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M4" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N4" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P4" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:16">
+    </x:row>
+    <x:row r="5" spans="1:17">
       <x:c r="A5" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
+      <x:c r="F5" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="P5" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
+      <x:c r="Q5" s="0" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="F5" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="G5" s="0" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="I5" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J5" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="K5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L5" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M5" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N5" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P5" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:16">
+    </x:row>
+    <x:row r="6" spans="1:17">
       <x:c r="A6" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
+      <x:c r="F6" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="P6" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s">
+      <x:c r="Q6" s="0" t="s">
         <x:v>35</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G6" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I6" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J6" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L6" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M6" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N6" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P6" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:16">
-      <x:c r="A7" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F7" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G7" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I7" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J7" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K7" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L7" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M7" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N7" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P7" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:16">
-      <x:c r="A8" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F8" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G8" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="H8" s="2" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="I8" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J8" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K8" s="0">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="L8" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M8" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N8" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P8" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:16">
-      <x:c r="A9" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F9" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G9" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="H9" s="2" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="I9" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J9" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K9" s="0">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="L9" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M9" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N9" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P9" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:16">
-      <x:c r="A10" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F10" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G10" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I10" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J10" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="K10" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L10" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M10" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N10" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P10" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:16">
-      <x:c r="A11" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D11" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E11" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F11" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G11" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I11" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J11" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="K11" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L11" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M11" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N11" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P11" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:16">
-      <x:c r="A12" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B12" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C12" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D12" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E12" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F12" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G12" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="H12" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="I12" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J12" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="K12" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L12" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M12" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N12" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P12" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:16">
-      <x:c r="A13" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B13" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C13" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D13" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E13" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="F13" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G13" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="H13" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="I13" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J13" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="K13" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="L13" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M13" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N13" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P13" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:16">
-      <x:c r="A14" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B14" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C14" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D14" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E14" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F14" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G14" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I14" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J14" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K14" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L14" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M14" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N14" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P14" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" spans="1:16">
-      <x:c r="A15" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B15" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C15" s="0" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D15" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E15" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F15" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G15" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I15" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="J15" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="K15" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L15" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="M15" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="N15" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="P15" s="0" t="s">
-        <x:v>14</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>